<commit_message>
robo de nfs atualizacao
</commit_message>
<xml_diff>
--- a/src/planilha/planilha_nfse.xlsx
+++ b/src/planilha/planilha_nfse.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="47">
   <si>
     <t xml:space="preserve">dataEmissao</t>
   </si>
@@ -155,6 +155,9 @@
   </si>
   <si>
     <t xml:space="preserve">MG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAMPINAS</t>
   </si>
   <si>
     <t xml:space="preserve">SERVICO DE FUNDACAO - TRADO MECANIZADO S</t>
@@ -171,7 +174,7 @@
     <numFmt numFmtId="167" formatCode="#,##0.00"/>
     <numFmt numFmtId="168" formatCode="#,##0.0000"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -198,6 +201,11 @@
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -255,7 +263,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -281,6 +289,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -677,10 +689,10 @@
     </row>
     <row r="2" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="n">
-        <v>46077</v>
+        <v>46083</v>
       </c>
       <c r="B2" s="4" t="n">
-        <v>46077</v>
+        <v>46083</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>34</v>
@@ -718,53 +730,53 @@
       <c r="Q2" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="R2" s="6" t="n">
-        <v>3201308</v>
-      </c>
-      <c r="S2" s="6" t="n">
-        <v>3201308</v>
-      </c>
-      <c r="T2" s="6" t="n">
-        <v>3201308</v>
-      </c>
-      <c r="U2" s="7" t="n">
+      <c r="R2" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="S2" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="T2" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="U2" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="V2" s="7" t="n">
+      <c r="V2" s="8" t="n">
         <v>0</v>
       </c>
       <c r="W2" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="X2" s="7" t="n">
+        <v>46</v>
+      </c>
+      <c r="X2" s="8" t="n">
         <v>0.95</v>
       </c>
-      <c r="Y2" s="7" t="n">
+      <c r="Y2" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="Z2" s="7" t="n">
+      <c r="Z2" s="8" t="n">
         <v>7.02</v>
       </c>
-      <c r="AA2" s="7" t="s">
+      <c r="AA2" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="AB2" s="7"/>
-      <c r="AC2" s="8" t="n">
+      <c r="AB2" s="8"/>
+      <c r="AC2" s="9" t="n">
         <v>4.76</v>
       </c>
-      <c r="AD2" s="7" t="n">
+      <c r="AD2" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="AE2" s="7" t="n">
+      <c r="AE2" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="AF2" s="7" t="n">
+      <c r="AF2" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="AG2" s="7" t="n">
+      <c r="AG2" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="AH2" s="7" t="n">
+      <c r="AH2" s="8" t="n">
         <v>369.26</v>
       </c>
     </row>

</xml_diff>

<commit_message>
criacao do fluxo que verifica o status de uploadplanilha
</commit_message>
<xml_diff>
--- a/src/planilha/planilha_nfse.xlsx
+++ b/src/planilha/planilha_nfse.xlsx
@@ -174,7 +174,7 @@
     <numFmt numFmtId="167" formatCode="#,##0.00"/>
     <numFmt numFmtId="168" formatCode="#,##0.0000"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -201,11 +201,6 @@
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -263,7 +258,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -289,10 +284,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -689,10 +680,10 @@
     </row>
     <row r="2" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="n">
-        <v>46083</v>
+        <v>46082</v>
       </c>
       <c r="B2" s="4" t="n">
-        <v>46083</v>
+        <v>46082</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>34</v>
@@ -730,53 +721,53 @@
       <c r="Q2" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="R2" s="7" t="s">
+      <c r="R2" s="6" t="s">
         <v>45</v>
       </c>
       <c r="S2" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="T2" s="7" t="s">
+      <c r="T2" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="U2" s="8" t="n">
+      <c r="U2" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="V2" s="8" t="n">
+      <c r="V2" s="7" t="n">
         <v>0</v>
       </c>
       <c r="W2" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="X2" s="8" t="n">
+      <c r="X2" s="7" t="n">
         <v>0.95</v>
       </c>
-      <c r="Y2" s="8" t="n">
+      <c r="Y2" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="Z2" s="8" t="n">
+      <c r="Z2" s="7" t="n">
         <v>7.02</v>
       </c>
-      <c r="AA2" s="8" t="s">
+      <c r="AA2" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="AB2" s="8"/>
-      <c r="AC2" s="9" t="n">
+      <c r="AB2" s="7"/>
+      <c r="AC2" s="8" t="n">
         <v>4.76</v>
       </c>
-      <c r="AD2" s="8" t="n">
+      <c r="AD2" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="AE2" s="8" t="n">
+      <c r="AE2" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="AF2" s="8" t="n">
+      <c r="AF2" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="AG2" s="8" t="n">
+      <c r="AG2" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="AH2" s="8" t="n">
+      <c r="AH2" s="7" t="n">
         <v>369.26</v>
       </c>
     </row>

</xml_diff>